<commit_message>
New skills (Chilli, Ice Arrow, Twin Shot, Volley, Bolts), unified Fork/Trident/Pitchfork, Crab Claws, one-off tags; recommended skill curriculum sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R6XsJCmXvcJWh931mAnv4Q
</commit_message>
<xml_diff>
--- a/docs/skills-by-map-2026-10-15.xlsx
+++ b/docs/skills-by-map-2026-10-15.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per skill" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unused &amp; unshown" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommended" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per skill" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unused &amp; unshown" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Per map'!$A$1:$H$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Per skill'!$A$1:$I$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unused &amp; unshown'!$A$1:$F$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Per map'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Per skill'!$A$1:$I$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Unused &amp; unshown'!$A$1:$F$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="003B5B3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E7C9"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -77,6 +83,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -503,6 +512,1341 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Map</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Biome / feel</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Skills – definite (new here)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Skills – maybe</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Shown first here today (for comparison)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Map 0</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Bramblewood Outskirts</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Meadow, misty (no day/night)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Flying, Swarm (ants only), Regeneration (Earthworm)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>0-4 boss: Thorns (its one new skill)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Flying, Armor, Swarm, Poison, trigger:onAttack, Tide, Quick, Worthy, Nocturnal, Stealth, Guardian</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Your call: only these three. Base bees don't swarm; pack 1 brings swarming bees. Your published Earthworm has no Regeneration yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Map 0 side</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tutorial</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Tutorial</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>(none new: reuse Map 0's three)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Dynamite, Helmet, bounty, Dry, Thorns, trigger:onKill, Swimmer, Diurnal, Fork, Worship, Prayer, freeze, trigger:onSpawn, Expose, Landslide, Arrow, Reload</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Today its optional fights show 17 skills (Dynamite, Helmet, Fork, Freeze, Prayer…). Trim these decks to Map 0's skills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Map 0 side</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>The Old Bramble</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Old forest</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Thorns</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Armor (snail)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Bleed</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Side maps: about 2 new skills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Map 1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Thistlewood</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Wet forest, day/night begins</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Diurnal, Nocturnal, Swarm on bees</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Rainrunner (the main Frog: bonus when raining), Quick</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Demolisher, Darksight, Keen Sense, Cleave, Twin Strike</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Day and night arrive together, so both phase skills land here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Map 1 side</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Clovermead</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Flower meadow</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Evasive (butterflies)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Bloom (flowers)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Evasive</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Map 2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Pebble Beach</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Shore</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Tide, Swimmer</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Shell/Armor (crabs), Crab Claws</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Molting, Wave, trigger:onReady, Revivificated</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Tide is revealed here (the '?' lifts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Map 2 side</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Lilypad Reach</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Pond</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Pounce (frogs)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Pounce, Healing, onReadyGold, Reach</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Map 2 side</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Smugglers' Grotto</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sea cave (Pitch Black)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Darksight, Lantern</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>shock, Electricity</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Darkness is a field effect from here on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Map 3</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Gannet Cliffs</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Sea cliffs</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Arrow, Skyfall</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Daunt</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Skyfall, onReadyDamage, Daunt</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>The first ranged skill: birds dive and shoot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Map 4</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Sunken Hollow</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Flooded lowland (Nest)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Armor, Thorns</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Gash, Inspiring</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Gash, Inspiring, Momentum</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>The Nest opens here: eggs and hatching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Map 5</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Gatorback Swamp</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Swamp</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Poison, Ambush</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Shedding, Explode</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Shedding, Regeneration, Ambush, explode</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Map 5 side</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>The Sunken Grove</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Swamp grove</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Healing (swamp medicine)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Poison Bolt</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Map 6</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Sable Swampmire</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Night swamp</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Bleed, Bloom (algae/fungal)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Fester, Remember</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Fester, Remember, trigger:onDeath, trigger:onAllyDie, Render</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Your 'Heal in the swamp maps' lands on Maps 5–6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Map 7</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>The Morel Hollow</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Fungi</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Sleep (spores), Decay</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Sprout/Growth</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>sleep, Decay, onDeathSpawn, Rocket</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Map 7 side</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>The Mycelium Deep</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Fungal dark</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Darkness (field)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Acid Bolt</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Earthquake, Brood</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Map 8</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Caves &amp; Alcoves</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Caves (Darkness)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Keen Sense, Electricity</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Shock Bolt, Stealth</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>sap, Shell</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>The electric bats live here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Map 8 side</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>The Glimmer Depths</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Crystal cave</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Shock</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Reflect</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Map 9</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>The Kelp Mangroves</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Wave, Molting</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Pierce, Twin</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Map 10</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Coral Current</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Reef</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Shell, Bloom (coral)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Moonpull</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Map 10 side</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>The Sunken Depths</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Deep sea (Darkness)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Moonpull</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Ice Bolt</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Corrode</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Map 11</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Eyrie Heights</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Mountain birds</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Volley, Twin Shot</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Swift, Snipe</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Midas Touch, Satiety, Lightning, Divine Retribution</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>The ranged family grows: Arrow → Twin Shot → Volley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Map 11 side</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>The Aerie Vault</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Mountain hall</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Snipe</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Map 12</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>The Briar Maze</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Bramble maze</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Sweep (cleave), Expose</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Backstab</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Keen Eye, Backstab, Snipe</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Map 13</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>The Redwood Deep</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Giant forest</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Guardian, Rage</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Demolisher, Boomerang</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Rage, King Slayer</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Map 14</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Savanna Reaches</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Savanna</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Pack / Pack Leader, Overwhelm</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Charge, Scare</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Bananarang, Durian, Stampede, Siege</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Map 14 side</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>The Canopy</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Jungle canopy</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Boomerang</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Evasive</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Bulwark</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Map 15</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>The Long Grass</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Tall grass</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Stealth, Pounce</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Backstab</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Map 16</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>The Pinewood Taiga</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Taiga</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Frostbite, Ice Arrow</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Lumberjack, Timber</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Map 17</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Wolfsbane Tundra</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Tundra</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Freeze, Ice Bolt</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Lone Wolf</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Frostbite, Lone Wolf</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Map 17 side</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>The Ice Hollow</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Ice cave</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Map 18</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>The Glass Dunes</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Desert</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Dry, Fire Bolt</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Changeling (mirage)</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Swift, Sociable, Fencing</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Map 19</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Ashen Spurn</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Ash slopes</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Fire Arrow, Immolation</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Heavy Metal</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Scare, Sacrifice</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Map 19 side</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Basalt Foundry</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Forge</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Siege, Helmet</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Dynamite, Rock Solid</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Stun, Frenzy, renewal, Fire Arrow, Pierce, scar, Immolation, grit, onSpawnDevilry, devour, Pitchfork, Desecrate, beware, ritual</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Map 20</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>The Sundered Peak</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Volcano peak</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Landslide, Lightning</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Supreme (dragons later)</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Maps 20–40: special, still no magic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Map 20 side</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Eye of the Volcano</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Crater</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Immolation</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Map 20 side</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Volcano Lair</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Lair</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Map 21</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>The Quiet Summit</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Summit (soft intro to 20–40)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Fencing, Counterattack</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Maps 50+</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Magic and weird stuff</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Magic, Ghost, Shade, Shadow, Psychic</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Irradiated, Ichor, Wither, Dragon Lightning</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Your rule: no magic before Map 50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>One-offs (any map)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Animal-specific, not tied to a map</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Coffee, Chilli, Banana, Bananarang, Durian, Rabid, Supreme Tide, Smoke Bomb, Avalanche, Earthquake, Tornado, Crepuscular, Scatterbrained, Meteor</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Hurricane (doesn't exist yet), Tsunami, Fireball</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Each lives on one animal; put them wherever that animal lives.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1895,7 +3239,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9616,7 +10960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>